<commit_message>
Qualify native Excel save and reopen of Numbers table borders
</commit_message>
<xml_diff>
--- a/OfficeIMO.TestAssets/Documents/IWorkCorpus/native-exports/numbers-table-borders-officeimo.xlsx
+++ b/OfficeIMO.TestAssets/Documents/IWorkCorpus/native-exports/numbers-table-borders-officeimo.xlsx
@@ -694,9 +694,7 @@
       <c r="C3" s="108" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="106" t="str">
-        <v/>
-      </c>
+      <c r="D3" s="106"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="109" t="s">

</xml_diff>